<commit_message>
eval logic update to grade /ritonavir suffixes leniently
</commit_message>
<xml_diff>
--- a/eval/error_analysis/analysis_by_qid.xlsx
+++ b/eval/error_analysis/analysis_by_qid.xlsx
@@ -21669,7 +21669,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -21685,7 +21685,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -21693,7 +21693,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -21701,7 +21701,7 @@
         </is>
       </c>
       <c r="L48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
@@ -21717,7 +21717,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -21725,7 +21725,7 @@
         </is>
       </c>
       <c r="R48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -25337,7 +25337,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M100" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
updated list eval logic
</commit_message>
<xml_diff>
--- a/eval/error_analysis/analysis_by_qid.xlsx
+++ b/eval/error_analysis/analysis_by_qid.xlsx
@@ -9531,7 +9531,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -9761,7 +9761,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -9769,7 +9769,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9793,7 +9793,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -9801,7 +9801,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -10139,7 +10139,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -10213,7 +10213,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -10229,7 +10229,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -10493,7 +10493,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -10509,7 +10509,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -10689,7 +10689,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -10829,7 +10829,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -11463,7 +11463,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -12055,7 +12055,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -12383,7 +12383,7 @@
         </is>
       </c>
       <c r="R40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -12409,7 +12409,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -12417,7 +12417,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -12425,7 +12425,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12449,7 +12449,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -12457,7 +12457,7 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -12837,7 +12837,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -12845,7 +12845,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -12861,7 +12861,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -12893,7 +12893,7 @@
         </is>
       </c>
       <c r="R47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -13231,7 +13231,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -13255,7 +13255,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
@@ -13263,7 +13263,7 @@
         </is>
       </c>
       <c r="R52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -13305,7 +13305,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -13329,7 +13329,7 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
@@ -13445,7 +13445,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="n">
@@ -13481,7 +13481,7 @@
         </is>
       </c>
       <c r="R55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -13663,7 +13663,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -13671,7 +13671,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -13695,7 +13695,7 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
@@ -13703,7 +13703,7 @@
         </is>
       </c>
       <c r="R58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -13819,7 +13819,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -13869,7 +13869,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -13893,7 +13893,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -13901,7 +13901,7 @@
         </is>
       </c>
       <c r="L61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -14091,7 +14091,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -14107,7 +14107,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -14139,7 +14139,7 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -14543,7 +14543,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -14551,7 +14551,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -14575,7 +14575,7 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
@@ -14583,7 +14583,7 @@
         </is>
       </c>
       <c r="R70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -14695,7 +14695,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -14719,7 +14719,7 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
@@ -14727,7 +14727,7 @@
         </is>
       </c>
       <c r="R72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -14835,7 +14835,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -14843,7 +14843,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -14859,7 +14859,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -14867,7 +14867,7 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
@@ -14875,7 +14875,7 @@
         </is>
       </c>
       <c r="R74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -15843,7 +15843,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -15851,7 +15851,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -15867,7 +15867,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -15933,7 +15933,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -15965,7 +15965,7 @@
         </is>
       </c>
       <c r="P89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
@@ -16089,7 +16089,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -16607,7 +16607,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -16739,7 +16739,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -16747,7 +16747,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
@@ -16755,7 +16755,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -16771,7 +16771,7 @@
         </is>
       </c>
       <c r="N100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -16779,7 +16779,7 @@
         </is>
       </c>
       <c r="P100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
@@ -16787,7 +16787,7 @@
         </is>
       </c>
       <c r="R100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -17071,7 +17071,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -17079,7 +17079,7 @@
         </is>
       </c>
       <c r="R104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -17607,7 +17607,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -18055,7 +18055,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -18063,7 +18063,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
@@ -18079,7 +18079,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -18087,7 +18087,7 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -18095,7 +18095,7 @@
         </is>
       </c>
       <c r="P118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
@@ -18103,7 +18103,7 @@
         </is>
       </c>
       <c r="R118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -19075,7 +19075,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -19107,7 +19107,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -19281,7 +19281,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -19297,7 +19297,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -19783,7 +19783,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -19915,7 +19915,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
@@ -19927,7 +19927,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -20059,7 +20059,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -20289,7 +20289,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -20347,7 +20347,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -20355,7 +20355,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -20379,7 +20379,7 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -20387,7 +20387,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -20395,7 +20395,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -20507,7 +20507,7 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -20619,7 +20619,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -20627,7 +20627,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -21471,7 +21471,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -21495,7 +21495,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
@@ -21503,7 +21503,7 @@
         </is>
       </c>
       <c r="N45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -21519,7 +21519,7 @@
         </is>
       </c>
       <c r="R45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -21595,7 +21595,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -21603,7 +21603,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -21627,7 +21627,7 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
@@ -21635,7 +21635,7 @@
         </is>
       </c>
       <c r="N47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -21669,7 +21669,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -21677,7 +21677,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -21953,7 +21953,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -21985,7 +21985,7 @@
         </is>
       </c>
       <c r="N52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -22715,7 +22715,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -22813,7 +22813,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -22863,7 +22863,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -22887,7 +22887,7 @@
         </is>
       </c>
       <c r="L65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -22999,7 +22999,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
@@ -23015,7 +23015,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -23517,7 +23517,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -23549,7 +23549,7 @@
         </is>
       </c>
       <c r="R74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -23575,7 +23575,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -23591,7 +23591,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -23599,7 +23599,7 @@
         </is>
       </c>
       <c r="L75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -23703,7 +23703,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -23711,7 +23711,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -23735,7 +23735,7 @@
         </is>
       </c>
       <c r="L77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -23743,7 +23743,7 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -23751,7 +23751,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
@@ -23759,7 +23759,7 @@
         </is>
       </c>
       <c r="R77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -23785,7 +23785,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -23809,7 +23809,7 @@
         </is>
       </c>
       <c r="L78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
@@ -24461,7 +24461,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -24485,7 +24485,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -24501,7 +24501,7 @@
         </is>
       </c>
       <c r="N88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -24605,7 +24605,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -24613,7 +24613,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -24621,7 +24621,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -24637,7 +24637,7 @@
         </is>
       </c>
       <c r="L90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -24815,7 +24815,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -24823,7 +24823,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -24831,7 +24831,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -24855,7 +24855,7 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -25091,7 +25091,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -25609,7 +25609,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M104" t="inlineStr">
         <is>
@@ -25625,7 +25625,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -25659,7 +25659,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -26095,7 +26095,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -26161,7 +26161,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -26169,7 +26169,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -26185,7 +26185,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -26193,7 +26193,7 @@
         </is>
       </c>
       <c r="L112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -26243,7 +26243,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -26585,7 +26585,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -26593,7 +26593,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
@@ -26601,7 +26601,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -26609,7 +26609,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -26617,7 +26617,7 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -26633,7 +26633,7 @@
         </is>
       </c>
       <c r="R118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">

</xml_diff>

<commit_message>
forgot to run evals after code fix
</commit_message>
<xml_diff>
--- a/eval/error_analysis/analysis_by_qid.xlsx
+++ b/eval/error_analysis/analysis_by_qid.xlsx
@@ -9917,7 +9917,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -10139,7 +10139,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -10213,7 +10213,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -12055,7 +12055,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -16089,7 +16089,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -16607,7 +16607,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -19075,7 +19075,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -19107,7 +19107,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -19281,7 +19281,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -19783,7 +19783,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -20289,7 +20289,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -20507,7 +20507,7 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -20619,7 +20619,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -20627,7 +20627,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -21471,7 +21471,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -21595,7 +21595,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -21635,7 +21635,7 @@
         </is>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -21985,7 +21985,7 @@
         </is>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -22501,7 +22501,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
@@ -22715,7 +22715,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -22813,7 +22813,7 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -22863,7 +22863,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -23015,7 +23015,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -23575,7 +23575,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -23591,7 +23591,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -23599,7 +23599,7 @@
         </is>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -23703,7 +23703,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -23711,7 +23711,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -23735,7 +23735,7 @@
         </is>
       </c>
       <c r="L77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -23743,7 +23743,7 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -23759,7 +23759,7 @@
         </is>
       </c>
       <c r="R77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -24485,7 +24485,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -24501,7 +24501,7 @@
         </is>
       </c>
       <c r="N88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -24605,7 +24605,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -24621,7 +24621,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -24637,7 +24637,7 @@
         </is>
       </c>
       <c r="L90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -24823,7 +24823,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -24855,7 +24855,7 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -25091,7 +25091,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -25609,7 +25609,7 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M104" t="inlineStr">
         <is>
@@ -25625,7 +25625,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -25659,7 +25659,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -26095,7 +26095,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -26169,7 +26169,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -26601,7 +26601,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -26609,7 +26609,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -26617,7 +26617,7 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -26633,7 +26633,7 @@
         </is>
       </c>
       <c r="R118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119">

</xml_diff>